<commit_message>
updated nitro-br+ complex coordinates
</commit_message>
<xml_diff>
--- a/depricated_examples/nitrobenzene/ortho_meta_orientation/QED_CCSD_(2,2)_Energies.xlsx
+++ b/depricated_examples/nitrobenzene/ortho_meta_orientation/QED_CCSD_(2,2)_Energies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jfoley19/Code/cqed-rhf/depricated_examples/nitrobenzene/ortho_meta_orientation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4891A8DE-89DE-BB42-A464-7F59D5D86C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83123EF4-3D33-F146-9069-F30BB4ECCC67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,10 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <t>Strong-Field Coupling — Intermediate Energies by Field Direction</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="29">
   <si>
     <t>Field
 Dir.</t>
@@ -84,6 +81,48 @@
   </si>
   <si>
     <t>Ez (unit vec.)</t>
+  </si>
+  <si>
+    <t>Jay's Reference (QED-CCSD(2,2)</t>
+  </si>
+  <si>
+    <t>Marcus QED-CCSD(2,0)</t>
+  </si>
+  <si>
+    <t>Marcus QED-CCSD(2,1)</t>
+  </si>
+  <si>
+    <t>Marcus QED-CCSD(2,2)</t>
+  </si>
+  <si>
+    <t>Ortho Energy Decomposition</t>
+  </si>
+  <si>
+    <t>canonical 1el energy</t>
+  </si>
+  <si>
+    <t>canonical 2el energy</t>
+  </si>
+  <si>
+    <t>bilinear coupling en</t>
+  </si>
+  <si>
+    <t>1-electron dse</t>
+  </si>
+  <si>
+    <t>2-electron dse</t>
+  </si>
+  <si>
+    <t>1-electron dipole dse</t>
+  </si>
+  <si>
+    <t>1-electron quadrupole dse</t>
+  </si>
+  <si>
+    <t>Para Energy Decomposition</t>
+  </si>
+  <si>
+    <t>Meta Energy Decomposition</t>
   </si>
 </sst>
 </file>
@@ -161,7 +200,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -184,11 +223,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -237,6 +285,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -539,19 +593,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="3" width="9" customWidth="1"/>
-    <col min="4" max="6" width="16" customWidth="1"/>
-    <col min="7" max="9" width="20" customWidth="1"/>
-    <col min="10" max="13" width="22" customWidth="1"/>
+    <col min="2" max="11" width="20.1640625" customWidth="1"/>
+    <col min="12" max="13" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="15" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -568,44 +620,44 @@
     </row>
     <row r="2" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="L2" s="14"/>
       <c r="M2" s="14"/>
     </row>
     <row r="3" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" s="3">
         <v>70.434782608695656</v>
@@ -640,7 +692,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="6">
         <v>70.434782608695656</v>
@@ -675,7 +727,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" s="9">
         <v>117.39130434782609</v>
@@ -710,7 +762,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" s="12">
         <v>62.608695652173907</v>
@@ -746,9 +798,742 @@
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="I8" s="17"/>
     </row>
+    <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.2">
+      <c r="A11" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="16"/>
+    </row>
+    <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L12" s="14"/>
+      <c r="M12" s="14"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="3">
+        <v>70.434782608695656</v>
+      </c>
+      <c r="C13" s="3">
+        <v>31.304347826086961</v>
+      </c>
+      <c r="D13" s="4">
+        <v>0.78781235979440856</v>
+      </c>
+      <c r="E13" s="4">
+        <v>0.55163215302282487</v>
+      </c>
+      <c r="F13" s="4">
+        <v>0.27395921869243262</v>
+      </c>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="6">
+        <v>70.434782608695656</v>
+      </c>
+      <c r="C14" s="6">
+        <v>156.52173913043481</v>
+      </c>
+      <c r="D14" s="7">
+        <v>-0.83289240593853064</v>
+      </c>
+      <c r="E14" s="7">
+        <v>0.48087065477460561</v>
+      </c>
+      <c r="F14" s="7">
+        <v>0.27395921869243262</v>
+      </c>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="9">
+        <v>117.39130434782609</v>
+      </c>
+      <c r="C15" s="9">
+        <v>156.52173913043481</v>
+      </c>
+      <c r="D15" s="10">
+        <v>-0.75000000000000011</v>
+      </c>
+      <c r="E15" s="10">
+        <v>0.4330127018922193</v>
+      </c>
+      <c r="F15" s="10">
+        <v>-0.49999999999999978</v>
+      </c>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A16" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" s="12">
+        <v>62.608695652173907</v>
+      </c>
+      <c r="C16" s="12">
+        <v>62.608695652173907</v>
+      </c>
+      <c r="D16" s="13">
+        <v>0.38302222155948901</v>
+      </c>
+      <c r="E16" s="13">
+        <v>0.82139380484326963</v>
+      </c>
+      <c r="F16" s="13">
+        <v>0.42261826174069939</v>
+      </c>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="13"/>
+      <c r="J16" s="13"/>
+      <c r="K16" s="13"/>
+    </row>
+    <row r="21" spans="1:13" ht="18" x14ac:dyDescent="0.2">
+      <c r="A21" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="16"/>
+    </row>
+    <row r="22" spans="1:13" ht="30" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L22" s="14"/>
+      <c r="M22" s="14"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B23" s="3">
+        <v>70.434782608695656</v>
+      </c>
+      <c r="C23" s="3">
+        <v>31.304347826086961</v>
+      </c>
+      <c r="D23" s="4">
+        <v>0.78781235979440856</v>
+      </c>
+      <c r="E23" s="4">
+        <v>0.55163215302282487</v>
+      </c>
+      <c r="F23" s="4">
+        <v>0.27395921869243262</v>
+      </c>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A24" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="6">
+        <v>70.434782608695656</v>
+      </c>
+      <c r="C24" s="6">
+        <v>156.52173913043481</v>
+      </c>
+      <c r="D24" s="7">
+        <v>-0.83289240593853064</v>
+      </c>
+      <c r="E24" s="7">
+        <v>0.48087065477460561</v>
+      </c>
+      <c r="F24" s="7">
+        <v>0.27395921869243262</v>
+      </c>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="7"/>
+      <c r="K24" s="7"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A25" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" s="9">
+        <v>117.39130434782609</v>
+      </c>
+      <c r="C25" s="9">
+        <v>156.52173913043481</v>
+      </c>
+      <c r="D25" s="10">
+        <v>-0.75000000000000011</v>
+      </c>
+      <c r="E25" s="10">
+        <v>0.4330127018922193</v>
+      </c>
+      <c r="F25" s="10">
+        <v>-0.49999999999999978</v>
+      </c>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A26" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B26" s="12">
+        <v>62.608695652173907</v>
+      </c>
+      <c r="C26" s="12">
+        <v>62.608695652173907</v>
+      </c>
+      <c r="D26" s="13">
+        <v>0.38302222155948901</v>
+      </c>
+      <c r="E26" s="13">
+        <v>0.82139380484326963</v>
+      </c>
+      <c r="F26" s="13">
+        <v>0.42261826174069939</v>
+      </c>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
+    </row>
+    <row r="30" spans="1:13" ht="18" x14ac:dyDescent="0.2">
+      <c r="A30" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="16"/>
+      <c r="I30" s="16"/>
+      <c r="J30" s="16"/>
+      <c r="K30" s="16"/>
+      <c r="L30" s="16"/>
+      <c r="M30" s="16"/>
+    </row>
+    <row r="31" spans="1:13" ht="30" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L31" s="14"/>
+      <c r="M31" s="14"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B32" s="3">
+        <v>70.434782608695656</v>
+      </c>
+      <c r="C32" s="3">
+        <v>31.304347826086961</v>
+      </c>
+      <c r="D32" s="4">
+        <v>0.78781235979440856</v>
+      </c>
+      <c r="E32" s="4">
+        <v>0.55163215302282487</v>
+      </c>
+      <c r="F32" s="4">
+        <v>0.27395921869243262</v>
+      </c>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A33" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B33" s="6">
+        <v>70.434782608695656</v>
+      </c>
+      <c r="C33" s="6">
+        <v>156.52173913043481</v>
+      </c>
+      <c r="D33" s="7">
+        <v>-0.83289240593853064</v>
+      </c>
+      <c r="E33" s="7">
+        <v>0.48087065477460561</v>
+      </c>
+      <c r="F33" s="7">
+        <v>0.27395921869243262</v>
+      </c>
+      <c r="G33" s="7"/>
+      <c r="H33" s="7"/>
+      <c r="I33" s="7"/>
+      <c r="J33" s="7"/>
+      <c r="K33" s="7"/>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A34" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34" s="9">
+        <v>117.39130434782609</v>
+      </c>
+      <c r="C34" s="9">
+        <v>156.52173913043481</v>
+      </c>
+      <c r="D34" s="10">
+        <v>-0.75000000000000011</v>
+      </c>
+      <c r="E34" s="10">
+        <v>0.4330127018922193</v>
+      </c>
+      <c r="F34" s="10">
+        <v>-0.49999999999999978</v>
+      </c>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
+      <c r="J34" s="10"/>
+      <c r="K34" s="10"/>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A35" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B35" s="12">
+        <v>62.608695652173907</v>
+      </c>
+      <c r="C35" s="12">
+        <v>62.608695652173907</v>
+      </c>
+      <c r="D35" s="13">
+        <v>0.38302222155948901</v>
+      </c>
+      <c r="E35" s="13">
+        <v>0.82139380484326963</v>
+      </c>
+      <c r="F35" s="13">
+        <v>0.42261826174069939</v>
+      </c>
+      <c r="G35" s="13"/>
+      <c r="H35" s="13"/>
+      <c r="I35" s="13"/>
+      <c r="J35" s="13"/>
+      <c r="K35" s="13"/>
+    </row>
+    <row r="39" spans="1:13" ht="18" x14ac:dyDescent="0.2">
+      <c r="A39" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B39" s="19"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="19"/>
+      <c r="F39" s="19"/>
+      <c r="G39" s="19"/>
+      <c r="H39" s="19"/>
+      <c r="I39" s="18"/>
+      <c r="J39" s="18"/>
+      <c r="K39" s="18"/>
+      <c r="L39" s="18"/>
+      <c r="M39" s="18"/>
+    </row>
+    <row r="40" spans="1:13" ht="30" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I40" s="14"/>
+      <c r="J40" s="14"/>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4"/>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A42" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B42" s="6"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="7"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="7"/>
+      <c r="G42" s="7"/>
+      <c r="H42" s="7"/>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A43" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B43" s="9"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A44" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B44" s="12"/>
+      <c r="C44" s="12"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="13"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="13"/>
+      <c r="H44" s="13"/>
+    </row>
+    <row r="49" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+      <c r="A49" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B49" s="19"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+      <c r="F49" s="19"/>
+      <c r="G49" s="19"/>
+      <c r="H49" s="19"/>
+    </row>
+    <row r="50" spans="1:8" ht="30" x14ac:dyDescent="0.2">
+      <c r="A50" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H50" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4"/>
+      <c r="G51" s="4"/>
+      <c r="H51" s="4"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A52" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B52" s="6"/>
+      <c r="C52" s="6"/>
+      <c r="D52" s="7"/>
+      <c r="E52" s="7"/>
+      <c r="F52" s="7"/>
+      <c r="G52" s="7"/>
+      <c r="H52" s="7"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A53" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B53" s="9"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="10"/>
+      <c r="E53" s="10"/>
+      <c r="F53" s="10"/>
+      <c r="G53" s="10"/>
+      <c r="H53" s="10"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A54" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B54" s="12"/>
+      <c r="C54" s="12"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="13"/>
+      <c r="F54" s="13"/>
+      <c r="G54" s="13"/>
+      <c r="H54" s="13"/>
+    </row>
+    <row r="59" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+      <c r="A59" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B59" s="19"/>
+      <c r="C59" s="19"/>
+      <c r="D59" s="19"/>
+      <c r="E59" s="19"/>
+      <c r="F59" s="19"/>
+      <c r="G59" s="19"/>
+      <c r="H59" s="19"/>
+    </row>
+    <row r="60" spans="1:8" ht="30" x14ac:dyDescent="0.2">
+      <c r="A60" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B61" s="3"/>
+      <c r="C61" s="3"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4"/>
+      <c r="F61" s="4"/>
+      <c r="G61" s="4"/>
+      <c r="H61" s="4"/>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A62" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B62" s="6"/>
+      <c r="C62" s="6"/>
+      <c r="D62" s="7"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="7"/>
+      <c r="G62" s="7"/>
+      <c r="H62" s="7"/>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A63" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B63" s="9"/>
+      <c r="C63" s="9"/>
+      <c r="D63" s="10"/>
+      <c r="E63" s="10"/>
+      <c r="F63" s="10"/>
+      <c r="G63" s="10"/>
+      <c r="H63" s="10"/>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A64" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B64" s="12"/>
+      <c r="C64" s="12"/>
+      <c r="D64" s="13"/>
+      <c r="E64" s="13"/>
+      <c r="F64" s="13"/>
+      <c r="G64" s="13"/>
+      <c r="H64" s="13"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="7">
+    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A59:H59"/>
     <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A11:M11"/>
+    <mergeCell ref="A21:M21"/>
+    <mergeCell ref="A30:M30"/>
+    <mergeCell ref="A39:H39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>